<commit_message>
tune battery recharge and engine charge params
</commit_message>
<xml_diff>
--- a/Data Sheets/Entities.xlsx
+++ b/Data Sheets/Entities.xlsx
@@ -648,7 +648,7 @@
     <t>Engines, Diesel Engines</t>
   </si>
   <si>
-    <t>/Velocity +10, Noise = 0.0, FuelUsage = 0.0, EnergyUsage = -0.55, SmokeVisibility = 0.0, MaxGearChangeDelay = 7</t>
+    <t>/Velocity +10, Noise = 0.0, FuelUsage = 0.0, EnergyUsage = -1.0, SmokeVisibility = 0.0, MaxGearChangeDelay = 7</t>
   </si>
   <si>
     <t>Electric Engines</t>
@@ -657,7 +657,7 @@
     <t>Engines, Electric Engines</t>
   </si>
   <si>
-    <t>/Velocity +10, Noise = 0.0, FuelUsage = -10.0, EnergyUsage = 0.0, MaxGearChangeDelay = 7</t>
+    <t>/Velocity +10, Noise = 0.0, FuelUsage = -1.0, EnergyUsage = 0.0, MaxGearChangeDelay = 7</t>
   </si>
   <si>
     <t>Radio Room</t>

</xml_diff>

<commit_message>
tune 43U cadence and normalize 88mm magazine size
</commit_message>
<xml_diff>
--- a/Data Sheets/Entities.xlsx
+++ b/Data Sheets/Entities.xlsx
@@ -666,7 +666,7 @@
     <t>Artillery - 8.8 cm</t>
   </si>
   <si>
-    <t>Calibre = 88, Range = 12000, ReloadTime = 0.1, MagazineSize = 4, HorizontalRecoil = 0.0, MinVerticalRecoil = 0.0, MaxVerticalRecoil = 0.0, SeriesTimeOffset = 0, RecoilDuration = 0.23, RecoilRecovery = 0.2, RecoilGrowthRate = 1.0, RecoilRecoveryRate = 0.996</t>
+    <t>Calibre = 88, Range = 12000, ReloadTime = 0.1, MagazineSize = 1, HorizontalRecoil = 0.0, MinVerticalRecoil = 0.0, MaxVerticalRecoil = 0.0, SeriesTimeOffset = 0, RecoilDuration = 0.23, RecoilRecovery = 0.2, RecoilGrowthRate = 1.0, RecoilRecoveryRate = 0.996</t>
   </si>
   <si>
     <t>Gyrocompass</t>
@@ -753,7 +753,7 @@
     <t>43U</t>
   </si>
   <si>
-    <t>Calibre = 20, Range = 5000, ReloadTime = 0.1, MagazineSize = 120, HorizontalRecoil = 1, MinVerticalRecoil = -0.3, MaxVerticalRecoil = 0.7, SeriesTimeOffset = 0.1, RecoilDuration = 0.3, RecoilRecovery = 0.2, RecoilGrowthRate = 0.07, RecoilRecoveryRate = 0.99, SkippedShells = 3</t>
+    <t>Calibre = 20, Range = 5000, ReloadTime = 0.1, MagazineSize = 120, HorizontalRecoil = 1, MinVerticalRecoil = -0.3, MaxVerticalRecoil = 0.7, SeriesTimeOffset = 0.1, RecoilDuration = 0.3, RecoilRecovery = 0.2, RecoilGrowthRate = 0.07, RecoilRecoveryRate = 0.99, SkippedShells = 1</t>
   </si>
   <si>
     <t>Generic Gun - 2.0 cm</t>

</xml_diff>